<commit_message>
Mod: Create LoadFile endpoint
</commit_message>
<xml_diff>
--- a/API/test.xlsx
+++ b/API/test.xlsx
@@ -51,6 +51,9 @@
     <x:t>Вагоно-километры в месяц</x:t>
   </x:si>
   <x:si>
+    <x:t>Примечание</x:t>
+  </x:si>
+  <x:si>
     <x:t>2. Фактическое количество перевезенных пассажиров:</x:t>
   </x:si>
   <x:si>
@@ -87,31 +90,25 @@
     <x:t>Доходы, причитающиеся от субъектов, установивших льготы, руб.</x:t>
   </x:si>
   <x:si>
-    <x:t>6.26</x:t>
-  </x:si>
-  <x:si>
-    <x:t>6010/6009</x:t>
+    <x:t>4.26</x:t>
+  </x:si>
+  <x:si>
+    <x:t>6008/6007</x:t>
   </x:si>
   <x:si>
     <x:t>Донецк-Иловайск</x:t>
   </x:si>
   <x:si>
-    <x:t>19:50-21:19</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Донецк-Ясиноваатя</x:t>
-  </x:si>
-  <x:si>
-    <x:t>19:50-20:11</x:t>
-  </x:si>
-  <x:si>
-    <x:t>4.26</x:t>
-  </x:si>
-  <x:si>
-    <x:t>5.26</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Донецк-Ясиноватая</x:t>
+    <x:t>17:59-19:28</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ясиноватая-Иловайск</x:t>
+  </x:si>
+  <x:si>
+    <x:t>18:21-19:28</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Описание для 6008/6007</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -498,7 +495,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:J7"/>
+  <x:dimension ref="A1:K4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="6.710625" style="0" customWidth="1"/>
@@ -508,14 +505,15 @@
     <x:col min="6" max="6" width="18.710625" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="15.710625" style="0" customWidth="1"/>
     <x:col min="8" max="10" width="18.710625" style="0" customWidth="1"/>
+    <x:col min="11" max="11" width="50.710625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:10">
+    <x:row r="1" spans="1:11">
       <x:c r="A1" s="0" t="s">
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:10">
+    <x:row r="2" spans="1:11">
       <x:c r="A2" s="1" t="s">
         <x:v>1</x:v>
       </x:c>
@@ -546,22 +544,25 @@
       <x:c r="J2" s="1" t="s">
         <x:v>10</x:v>
       </x:c>
-    </x:row>
-    <x:row r="3" spans="1:10">
+      <x:c r="K2" s="1" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:11">
       <x:c r="A3" s="0">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="F3" s="0">
         <x:v>54</x:v>
@@ -573,143 +574,50 @@
         <x:v>216</x:v>
       </x:c>
       <x:c r="I3" s="0">
-        <x:v>0</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="J3" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:10">
+        <x:v>6264</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:11">
       <x:c r="A4" s="0">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>12</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G4" s="0">
         <x:v>4</x:v>
       </x:c>
       <x:c r="H4" s="0">
-        <x:v>48</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="I4" s="0">
-        <x:v>18</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="J4" s="0">
-        <x:v>864</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:10">
-      <x:c r="A5" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>23</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D5" s="0" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="E5" s="0" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="F5" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G5" s="0">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="H5" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I5" s="0">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="J5" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:10">
-      <x:c r="A6" s="0">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="K4" s="0" t="s">
         <x:v>30</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D6" s="0" t="s">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="E6" s="0" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="F6" s="0">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="G6" s="0">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="H6" s="0">
-        <x:v>216</x:v>
-      </x:c>
-      <x:c r="I6" s="0">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="J6" s="0">
-        <x:v>5616</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" spans="1:10">
-      <x:c r="A7" s="0">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="C7" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D7" s="0" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="E7" s="0" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="F7" s="0">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="G7" s="0">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="H7" s="0">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="I7" s="0">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="J7" s="0">
-        <x:v>240</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells count="1">
-    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A1:K1"/>
   </x:mergeCells>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
@@ -724,7 +632,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:M6"/>
+  <x:dimension ref="A1:M4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="6.710625" style="0" customWidth="1"/>
@@ -734,7 +642,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:13">
       <x:c r="A1" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:13">
@@ -745,17 +653,17 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C2" s="2" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D2" s="2" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="E2" s="2"/>
       <x:c r="F2" s="2"/>
       <x:c r="G2" s="2"/>
       <x:c r="H2" s="2"/>
       <x:c r="I2" s="2" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="J2" s="2"/>
       <x:c r="K2" s="2"/>
@@ -767,34 +675,34 @@
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
       <x:c r="D3" s="2" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E3" s="2" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="F3" s="2" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G3" s="2" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="H3" s="2" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="I3" s="2" t="s">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="F3" s="2" t="s">
+      <x:c r="J3" s="2" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="G3" s="2" t="s">
+      <x:c r="K3" s="2" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="H3" s="2" t="s">
+      <x:c r="L3" s="2" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="I3" s="2" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="J3" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="K3" s="2" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="L3" s="2" t="s">
-        <x:v>18</x:v>
-      </x:c>
       <x:c r="M3" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:13">
@@ -802,122 +710,40 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>44</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="E4" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>0</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H4" s="0">
-        <x:v>0</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="I4" s="0">
-        <x:v>12.202562538133</x:v>
+        <x:v>20.6017645728075</x:v>
       </x:c>
       <x:c r="J4" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="K4" s="0">
-        <x:v>0</x:v>
+        <x:v>20.8053691275168</x:v>
       </x:c>
       <x:c r="L4" s="0">
-        <x:v>0</x:v>
+        <x:v>12.751677852349</x:v>
       </x:c>
       <x:c r="M4" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:13">
-      <x:c r="A5" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D5" s="0">
-        <x:v>258</x:v>
-      </x:c>
-      <x:c r="E5" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F5" s="0">
-        <x:v>6</x:v>
-      </x:c>
-      <x:c r="G5" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H5" s="0">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="I5" s="0">
-        <x:v>17.2051402112273</x:v>
-      </x:c>
-      <x:c r="J5" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K5" s="0">
-        <x:v>24.3847874720358</x:v>
-      </x:c>
-      <x:c r="L5" s="0">
-        <x:v>53.6912751677852</x:v>
-      </x:c>
-      <x:c r="M5" s="0">
-        <x:v>12.751677852349</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:13">
-      <x:c r="A6" s="0">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D6" s="0">
-        <x:v>284</x:v>
-      </x:c>
-      <x:c r="E6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F6" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I6" s="0">
-        <x:v>14.7461952925607</x:v>
-      </x:c>
-      <x:c r="J6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K6" s="0">
-        <x:v>12.751677852349</x:v>
-      </x:c>
-      <x:c r="L6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M6" s="0">
-        <x:v>0</x:v>
+        <x:v>19.6999605211212</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -942,7 +768,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:L6"/>
+  <x:dimension ref="A1:L4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="6.710625" style="0" customWidth="1"/>
@@ -952,7 +778,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:12">
       <x:c r="A1" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>21</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:12">
@@ -963,17 +789,17 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C2" s="2" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D2" s="2" t="s">
-        <x:v>21</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E2" s="2"/>
       <x:c r="F2" s="2"/>
       <x:c r="G2" s="2"/>
       <x:c r="H2" s="2"/>
       <x:c r="I2" s="2" t="s">
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="J2" s="2"/>
       <x:c r="K2" s="2"/>
@@ -984,31 +810,31 @@
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
       <x:c r="D3" s="2" t="s">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E3" s="2" t="s">
-        <x:v>16</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="F3" s="2" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="G3" s="2" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="H3" s="2" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="I3" s="2" t="s">
         <x:v>17</x:v>
       </x:c>
-      <x:c r="G3" s="2" t="s">
+      <x:c r="J3" s="2" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="H3" s="2" t="s">
+      <x:c r="K3" s="2" t="s">
         <x:v>19</x:v>
       </x:c>
-      <x:c r="I3" s="2" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="J3" s="2" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="K3" s="2" t="s">
-        <x:v>18</x:v>
-      </x:c>
       <x:c r="L3" s="2" t="s">
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:12">
@@ -1016,113 +842,37 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>800</x:v>
+        <x:v>21856</x:v>
       </x:c>
       <x:c r="E4" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>0</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>0</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="H4" s="0">
-        <x:v>0</x:v>
+        <x:v>998</x:v>
       </x:c>
       <x:c r="I4" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="J4" s="0">
-        <x:v>0</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="K4" s="0">
         <x:v>0</x:v>
       </x:c>
       <x:c r="L4" s="0">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:12">
-      <x:c r="A5" s="0">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D5" s="0">
-        <x:v>6614</x:v>
-      </x:c>
-      <x:c r="E5" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F5" s="0">
-        <x:v>218</x:v>
-      </x:c>
-      <x:c r="G5" s="0">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="H5" s="0">
-        <x:v>19</x:v>
-      </x:c>
-      <x:c r="I5" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J5" s="0">
-        <x:v>218</x:v>
-      </x:c>
-      <x:c r="K5" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L5" s="0">
-        <x:v>19</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" spans="1:12">
-      <x:c r="A6" s="0">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="D6" s="0">
-        <x:v>6240</x:v>
-      </x:c>
-      <x:c r="E6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="I6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J6" s="0">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="K6" s="0">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="L6" s="0">
-        <x:v>0</x:v>
+        <x:v>998</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>